<commit_message>
[1 22] update ex1.py
</commit_message>
<xml_diff>
--- a/day1/sample.xlsx
+++ b/day1/sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -421,6 +421,38 @@
         <v>42</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>